<commit_message>
C14 influencer comment: push back with follower-distribution evidence
Per Mao's decision, no top-n% rerun. Quantified the asymmetry from our
data (TS top account 56x its own p99.9 vs 5x on Bluesky; top-8 share
16% vs 6%; TS #8 > Bluesky #1) and drafted the response paragraph into
the skeleton; tracker row updated.

Claude-Session: https://claude.ai/code/session_01V3T7pRg8oBYyTqLzP3YMYX
</commit_message>
<xml_diff>
--- a/paper/revision/reviewer_response_tracker.xlsx
+++ b/paper/revision/reviewer_response_tracker.xlsx
@@ -1041,22 +1041,22 @@
       </c>
       <c r="E15" s="1" t="inlineStr">
         <is>
-          <t>Rerun the influencer exclusion using the top 1, 5, and 10 percent most-followed accounts on both platforms and show the results hold; keep the original cutoff as one specification.</t>
+          <t>Push back with evidence rather than rerun. Our data show Truth Social has a separated influencer class that Bluesky lacks: the top TS account has 56 times the followers of the platform's 99.9th percentile account (Bluesky: 5 times), the top 8 TS accounts hold 16 percent of all follower ties (Bluesky: 6 percent), and TS's 8th account outranks Bluesky's 1st. A symmetric top-n-percent rule would remove ordinary accounts on one platform to mirror an anomaly on the other. Add these numbers to the appendix next to the follower CCDF.</t>
         </is>
       </c>
       <c r="F15" s="1" t="inlineStr">
         <is>
-          <t>Yes, small</t>
+          <t>Done (distribution stats computed)</t>
         </is>
       </c>
       <c r="G15" s="1" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Response paragraph drafted; appendix numbers ready</t>
         </is>
       </c>
       <c r="H15" s="1" t="inlineStr">
         <is>
-          <t>Half a day</t>
+          <t>Add the statistics to the appendix text</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Disambiguate tracker rows C1 (linking rule) vs C2 (follow-network timing)
Claude-Session: https://claude.ai/code/session_01V3T7pRg8oBYyTqLzP3YMYX
</commit_message>
<xml_diff>
--- a/paper/revision/reviewer_response_tracker.xlsx
+++ b/paper/revision/reviewer_response_tracker.xlsx
@@ -485,7 +485,7 @@
       </c>
       <c r="C2" s="1" t="inlineStr">
         <is>
-          <t>Repost cascades are reconstructed, not observed. The similarity between platforms could be an artifact of the reconstruction method. Validate it or drop reposts.</t>
+          <t>True repost paths are not observed, so we rebuild them by linking each repost to an earlier reposter the user follows. Reviewers worry that our choice of LINKING RULE could itself create the cross-platform similarity, and ask us to validate it or drop the repost analysis.</t>
         </is>
       </c>
       <c r="D2" s="1" t="inlineStr">
@@ -527,7 +527,7 @@
       </c>
       <c r="C3" s="1" t="inlineStr">
         <is>
-          <t>A user may have followed someone only after reposting, so inferred paths could be wrong. Could this error differ between platforms?</t>
+          <t>Different from C1: here the concern is the FOLLOW NETWORK we link with, not the linking rule. We collected who-follows-whom after the fact, so a follow edge we rely on may have been created only after the repost happened. R3 asks us to discuss this error and whether it differs between platforms.</t>
         </is>
       </c>
       <c r="D3" s="1" t="inlineStr">
@@ -537,7 +537,7 @@
       </c>
       <c r="E3" s="1" t="inlineStr">
         <is>
-          <t>Our follow networks have no timestamps, so we cannot check follow dates directly. We will add a sensitivity check that randomly deletes 5 to 30 percent of follow edges and shows the results hold, plus an honest limitation sentence noting the platform asymmetry in data collection.</t>
+          <t>Neither platform provides follow dates, so we cannot check the timing directly. We will run a sensitivity check that randomly deletes 5 to 30 percent of follow edges, simulating follows that did not exist yet at repost time, and show the results hold. We will also note the error has a known direction (a spurious follow edge can only move a repost from the root to deeper in the tree, a case already bounded by the C1 checks) and add a limitation sentence about the different crawl times of the two follow networks.</t>
         </is>
       </c>
       <c r="F3" s="1" t="inlineStr">

</xml_diff>

<commit_message>
Noise propagation complete: attenuation conclusion robust (C6)
Per-platform measured noise: all 100 draws keep >=83% of the baseline
platform divergence absorbed by ideology controls (median ~95%,
matching the unperturbed model). Pooled-matrix stress test: ~62-71%
absorbed. Classical attenuation direction means published estimates
are a lower bound. Results + caveats in results/noise_propagation/.

Claude-Session: https://claude.ai/code/session_01V3T7pRg8oBYyTqLzP3YMYX
</commit_message>
<xml_diff>
--- a/paper/revision/reviewer_response_tracker.xlsx
+++ b/paper/revision/reviewer_response_tracker.xlsx
@@ -715,12 +715,12 @@
       </c>
       <c r="G7" s="1" t="inlineStr">
         <is>
-          <t>Confusion matrices ready; simulation not started</t>
+          <t>DONE. All 100 draws under measured per-platform noise keep at least 83 percent of the platform gap absorbed (median 95 percent); a cruder pooled stress test still absorbs about two thirds. See results/noise_propagation/RESULTS.md</t>
         </is>
       </c>
       <c r="H7" s="1" t="inlineStr">
         <is>
-          <t>1 to 2 days</t>
+          <t>Write the appendix paragraph and add the summary table</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
C2 follow-timing sensitivity complete; all analysis items done
Deleting follow edges at random at 5 to 30 percent (simulating edges
that postdate the repost) moves the repost breadth interaction from
0.031 to 0.005 and depth from 0.004 to 0.013, an order of magnitude
below the reply values. Written into the appendix with an explicit
note that the error may be platform-asymmetric and that the test
bounds the consequence without measuring the true rate.

Tracker: 17 of 21 items complete. Outstanding are the annotation
top-up (needs Mao and Chen), the motif figure layout (needs a
notebook rerun), and optional further citations.

Claude-Session: https://claude.ai/code/session_01329QtyW5RwGQqnz6ETkQv4
</commit_message>
<xml_diff>
--- a/paper/revision/reviewer_response_tracker.xlsx
+++ b/paper/revision/reviewer_response_tracker.xlsx
@@ -537,22 +537,22 @@
       </c>
       <c r="E3" s="1" t="inlineStr">
         <is>
-          <t>Neither platform provides follow dates, so we cannot check the timing directly. We will run a sensitivity check that randomly deletes 5 to 30 percent of follow edges, simulating follows that did not exist yet at repost time, and show the results hold. We will also note the error has a known direction (a spurious follow edge can only move a repost from the root to deeper in the tree, a case already bounded by the C1 checks) and add a limitation sentence about the different crawl times of the two follow networks.</t>
+          <t>Neither platform exposes follow creation dates, so we cannot verify timing directly. We bound the consequence two ways. The error has a known direction: a follow that did not yet exist can only move a repost from the root to an interior parent, a displacement already covered by the alternative rules in C1. And we ran a direct test, deleting follow edges at random at 5 to 30 percent and re-estimating: the breadth interaction moves from 0.031 to 0.005 and depth from 0.004 to 0.013, both far below the reply values of 0.170 and -0.182. We also state that the error may be asymmetric, since the two follow networks were crawled at different times and Truth Social accounts have larger followee sets.</t>
         </is>
       </c>
       <c r="F3" s="1" t="inlineStr">
         <is>
-          <t>Yes, small</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="G3" s="1" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="H3" s="1" t="inlineStr">
         <is>
-          <t>Half a day: one loop over the existing robustness code</t>
+          <t>Written</t>
         </is>
       </c>
     </row>
@@ -1209,7 +1209,7 @@
       </c>
       <c r="E19" s="1" t="inlineStr">
         <is>
-          <t>Quality pass on every figure: labels, overlap, axis titles, consistent fonts and resolution.</t>
+          <t>Audited all 12 figures: every one is at or above 300 dpi, so resolution is fine. The real issue is in the two motif figures, where the family labels (Aligned, End shift, Mid shift, Diverse) are drawn as watermarks inside the plot and sit on top of the data, and where two families both show alignment = 0.00, which reads as an error. We clarified both captions now. Moving the labels above the axes requires re-running the notebook cell that builds the figure, which is the one presentation item still outstanding.</t>
         </is>
       </c>
       <c r="F19" s="1" t="inlineStr">
@@ -1219,12 +1219,12 @@
       </c>
       <c r="G19" s="1" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Partly done (captions fixed; layout needs a notebook rerun)</t>
         </is>
       </c>
       <c r="H19" s="1" t="inlineStr">
         <is>
-          <t>1 to 2 days</t>
+          <t>Half a day, needs the notebook environment</t>
         </is>
       </c>
     </row>
@@ -1293,7 +1293,7 @@
       </c>
       <c r="E21" s="1" t="inlineStr">
         <is>
-          <t>Notation pass (define at first use) and fix the indentation.</t>
+          <t>Fixed the stray indent (a blank line after display math started a new paragraph). Notation defined at first use in the revised sections.</t>
         </is>
       </c>
       <c r="F21" s="1" t="inlineStr">
@@ -1303,12 +1303,12 @@
       </c>
       <c r="G21" s="1" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="H21" s="1" t="inlineStr">
         <is>
-          <t>Hours</t>
+          <t>Written</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Mark C14 complete (appendix statistics already written)
Claude-Session: https://claude.ai/code/session_01329QtyW5RwGQqnz6ETkQv4
</commit_message>
<xml_diff>
--- a/paper/revision/reviewer_response_tracker.xlsx
+++ b/paper/revision/reviewer_response_tracker.xlsx
@@ -1051,12 +1051,12 @@
       </c>
       <c r="G15" s="1" t="inlineStr">
         <is>
-          <t>Response paragraph drafted; appendix numbers ready</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="H15" s="1" t="inlineStr">
         <is>
-          <t>Add the statistics to the appendix text</t>
+          <t>Written (appendix reports the distribution statistics; response paragraph drafted)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Write the validation defense into the paper, letter, and tracker
Defends the 200-item sample rather than extending it, per Mao:
directional test (significant on both platforms), invariance to which
annotator is the reference (with the harsher single-annotator rates
adopted as a worst case), and the post-to-user aggregation gain.
Removed all new-data language from the deliverables.

Claude-Session: https://claude.ai/code/session_01329QtyW5RwGQqnz6ETkQv4
</commit_message>
<xml_diff>
--- a/paper/revision/reviewer_response_tracker.xlsx
+++ b/paper/revision/reviewer_response_tracker.xlsx
@@ -463,7 +463,7 @@
       </c>
       <c r="G1" t="inlineStr">
         <is>
-          <t>Status (Aug 24)</t>
+          <t>Status (Aug 30)</t>
         </is>
       </c>
       <c r="H1" t="inlineStr">
@@ -621,7 +621,7 @@
       </c>
       <c r="E5" s="1" t="inlineStr">
         <is>
-          <t>Recomputed from the canonical file src/val_ideology.csv (an earlier run used a superseded copy whose second annotator differed on 15 items). Report per-class and per-platform precision and recall with percentile bootstrap 95 percent intervals over 2,000 resamples, plus overall accuracy 0.86 and inter-annotator kappa 0.77 [0.70, 0.85]. Per Ceren, we do NOT stratify-upsample the rare classes, since that invites the objection that the validation set was built to look good. The bootstrap shows exactly where the evidence is thin: pooled and majority-class rates are tight; right-on-Bluesky rests on 8 items with an interval of 0.33 to 0.91. Plan is to add a modest amount of unstratified annotation and show the rates do not move.</t>
+          <t>Defend the sample we have; collect nothing new. Every rate carries a percentile bootstrap interval, so a reader sees which cells are solid (pooled and majority classes) and which are thin (right-on-Bluesky, 8 items, 0.33 to 0.91). Three checks then establish what the sample does support: (a) the directional claim, that each platform's minority is over-assigned, is significant on both platforms (p = 0.017 and 0.004); (b) the pattern is unchanged whether we score against Annotator 1, Annotator 2, or consensus, and we adopt the harsher single-annotator rates as a worst case; (c) user labels aggregate multiple posts, so user-level accuracy (0.87 to 0.88) exceeds the post-level accuracy we validate (0.81 to 0.85), making the noise analysis conservative. Most directly, the noise analysis now includes a nested bootstrap that resamples the validation set itself, carrying its uncertainty into the substantive result.</t>
         </is>
       </c>
       <c r="F5" s="1" t="inlineStr">
@@ -631,12 +631,12 @@
       </c>
       <c r="G5" s="1" t="inlineStr">
         <is>
-          <t>Done (bootstrap reported); modest unstratified top-up planned</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="H5" s="1" t="inlineStr">
         <is>
-          <t>Optional: some more annotation, unstratified, to show rates are stable</t>
+          <t>Written</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update tracker and response letter for the motif figure fix (20/21 done)
Claude-Session: https://claude.ai/code/session_01329QtyW5RwGQqnz6ETkQv4
</commit_message>
<xml_diff>
--- a/paper/revision/reviewer_response_tracker.xlsx
+++ b/paper/revision/reviewer_response_tracker.xlsx
@@ -1209,7 +1209,7 @@
       </c>
       <c r="E19" s="1" t="inlineStr">
         <is>
-          <t>Audited all 12 figures: every one is at or above 300 dpi, so resolution is fine. The real issue is in the two motif figures, where the family labels (Aligned, End shift, Mid shift, Diverse) are drawn as watermarks inside the plot and sit on top of the data, and where two families both show alignment = 0.00, which reads as an error. We clarified both captions now. Moving the labels above the axes requires re-running the notebook cell that builds the figure, which is the one presentation item still outstanding.</t>
+          <t>Audited all 12 figures: every one is at or above 300 dpi. The substantive defect was in the two motif figures, where the family labels were drawn as watermarks inside the panel and sat on top of the data. Both figures are rebuilt with the labels in a header band above the axes, from a standalone script that reads the motif pipeline's z-score files, so they no longer depend on notebook state. Data, ordering, palette and thresholds unchanged; values spot-checked against the source files. Captions updated to match.</t>
         </is>
       </c>
       <c r="F19" s="1" t="inlineStr">
@@ -1219,12 +1219,12 @@
       </c>
       <c r="G19" s="1" t="inlineStr">
         <is>
-          <t>Partly done (captions fixed; layout needs a notebook rerun)</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="H19" s="1" t="inlineStr">
         <is>
-          <t>Half a day, needs the notebook environment</t>
+          <t>Written</t>
         </is>
       </c>
     </row>

</xml_diff>